<commit_message>
feat(masterdata): 경제 표에 연속 날갯짓 고비 코인 — combo_coins·판당 20·COMBO_REWARD 일일 300
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#EconomyConfig.xlsx
+++ b/table/Datas/#EconomyConfig.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,16 @@
           <t>daily_caps#sep=,</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>combo_per_match_max_coins</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>combo_coins#sep=,</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -539,6 +549,16 @@
           <t>list,ReasonCap</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>list,StatCoin</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -606,6 +626,16 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>daily_caps</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>combo_per_match_max_coins</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>combo_coins</t>
         </is>
       </c>
     </row>
@@ -642,7 +672,15 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>MATCH_REWARD,1,1500</t>
+          <t>MATCH_REWARD,1,1500,COMBO_REWARD,1,300</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>flapCombo10,2,flapCombo25,3,flapCombo50,5,flapCombo100,10</t>
         </is>
       </c>
     </row>

</xml_diff>